<commit_message>
cambiar piso por parada
</commit_message>
<xml_diff>
--- a/app/templates/solicitud_template.xlsx
+++ b/app/templates/solicitud_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t xml:space="preserve">MAPPING</t>
   </si>
@@ -34,13 +34,10 @@
     <t xml:space="preserve">Dirección</t>
   </si>
   <si>
-    <t xml:space="preserve">N° ascensores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N° Pisos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORREO</t>
+    <t xml:space="preserve">Nro ascensores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nro Paradas</t>
   </si>
 </sst>
 </file>
@@ -50,7 +47,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -81,16 +78,8 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
-    <font>
-      <u val="single"/>
-      <sz val="11"/>
-      <color rgb="FF0563C1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -101,12 +90,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFBFBFBF"/>
         <bgColor rgb="FFCCCCFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor rgb="FFFF9900"/>
       </patternFill>
     </fill>
   </fills>
@@ -140,7 +123,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -164,44 +147,40 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -227,7 +206,7 @@
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0563C1"/>
+      <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -248,7 +227,7 @@
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFC000"/>
+      <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
@@ -271,52 +250,57 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="27.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="28.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="27.42"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>6</v>
-      </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="5"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
     </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>